<commit_message>
Patients report for VN done
</commit_message>
<xml_diff>
--- a/api/templates/xpert_m4b1_patients/en.xlsx
+++ b/api/templates/xpert_m4b1_patients/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\xpert_m4b1_patients\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEFEC129-B4BC-46FF-BF06-D8B29537432A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0853380D-4218-4CF2-8012-16534167D580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0B124328-57BC-4FCF-919D-A7394F83025A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B124328-57BC-4FCF-919D-A7394F83025A}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="77">
   <si>
     <t xml:space="preserve">MINISTRY OF HEALTH </t>
   </si>
@@ -109,12 +109,6 @@
     <t>B</t>
   </si>
   <si>
-    <t>Smear ????</t>
-  </si>
-  <si>
-    <t>Other ????</t>
-  </si>
-  <si>
     <t>(1)=(2)+…+(9)</t>
   </si>
   <si>
@@ -273,6 +267,9 @@
   </si>
   <si>
     <t>Error (Error, No Result and Invalid MTB)</t>
+  </si>
+  <si>
+    <t>Trace</t>
   </si>
 </sst>
 </file>
@@ -511,7 +508,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -601,10 +598,130 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -613,128 +730,12 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -779,7 +780,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>1271120</xdr:colOff>
+          <xdr:colOff>1276350</xdr:colOff>
           <xdr:row>6</xdr:row>
           <xdr:rowOff>168275</xdr:rowOff>
         </xdr:to>
@@ -846,7 +847,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
-          <xdr:colOff>104588</xdr:colOff>
+          <xdr:colOff>114300</xdr:colOff>
           <xdr:row>6</xdr:row>
           <xdr:rowOff>168275</xdr:rowOff>
         </xdr:to>
@@ -1278,12 +1279,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="43" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
+      <c r="A1" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -1306,12 +1307,12 @@
       <c r="V1" s="3"/>
     </row>
     <row r="2" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -1332,22 +1333,22 @@
       <c r="V2" s="3"/>
     </row>
     <row r="3" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="45"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
       <c r="O3" s="4"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
@@ -1358,22 +1359,22 @@
       <c r="V3" s="3"/>
     </row>
     <row r="4" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="46" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="46"/>
-      <c r="L4" s="46"/>
-      <c r="M4" s="46"/>
-      <c r="N4" s="46"/>
+      <c r="A4" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="32"/>
+      <c r="M4" s="32"/>
+      <c r="N4" s="32"/>
       <c r="O4" s="5"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
@@ -1384,28 +1385,28 @@
       <c r="V4" s="3"/>
     </row>
     <row r="5" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
+      <c r="B5" s="33"/>
+      <c r="C5" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
       <c r="F5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="59" t="s">
-        <v>74</v>
-      </c>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="59"/>
-      <c r="M5" s="59"/>
-      <c r="N5" s="59"/>
+      <c r="G5" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="H5" s="34"/>
+      <c r="I5" s="34"/>
+      <c r="J5" s="34"/>
+      <c r="K5" s="34"/>
+      <c r="L5" s="34"/>
+      <c r="M5" s="34"/>
+      <c r="N5" s="34"/>
       <c r="O5" s="3"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
@@ -1416,32 +1417,32 @@
       <c r="V5" s="3"/>
     </row>
     <row r="6" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="37" t="s">
-        <v>73</v>
-      </c>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
       <c r="F6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="59" t="s">
-        <v>75</v>
-      </c>
-      <c r="H6" s="59"/>
-      <c r="I6" s="59"/>
+      <c r="G6" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
       <c r="J6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="K6" s="59" t="s">
-        <v>76</v>
-      </c>
-      <c r="L6" s="59"/>
-      <c r="M6" s="59"/>
-      <c r="N6" s="59"/>
+      <c r="K6" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="L6" s="34"/>
+      <c r="M6" s="34"/>
+      <c r="N6" s="34"/>
       <c r="O6" s="3"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="3"/>
@@ -1452,21 +1453,21 @@
       <c r="V6" s="3"/>
     </row>
     <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="37"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="33"/>
       <c r="D7" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="38" t="s">
+      <c r="G7" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="38"/>
-      <c r="I7" s="38"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="35"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
@@ -1482,28 +1483,28 @@
       <c r="V7" s="3"/>
     </row>
     <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="39"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="40" t="s">
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
-      <c r="K8" s="32"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="34" t="s">
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="40"/>
+      <c r="K8" s="40"/>
+      <c r="L8" s="40"/>
+      <c r="M8" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="N8" s="32" t="s">
+      <c r="N8" s="40" t="s">
         <v>16</v>
       </c>
       <c r="O8" s="8"/>
@@ -1516,30 +1517,30 @@
       <c r="V8" s="3"/>
     </row>
     <row r="9" spans="1:24" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="39"/>
-      <c r="B9" s="39"/>
-      <c r="C9" s="39"/>
-      <c r="D9" s="41"/>
-      <c r="E9" s="33" t="s">
+      <c r="A9" s="36"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="33" t="s">
+      <c r="F9" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33" t="s">
+      <c r="G9" s="41"/>
+      <c r="H9" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="33"/>
-      <c r="J9" s="33" t="s">
+      <c r="I9" s="41"/>
+      <c r="J9" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="33"/>
-      <c r="L9" s="33" t="s">
-        <v>77</v>
-      </c>
-      <c r="M9" s="35"/>
-      <c r="N9" s="32"/>
+      <c r="K9" s="41"/>
+      <c r="L9" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="M9" s="43"/>
+      <c r="N9" s="40"/>
       <c r="O9" s="8"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
@@ -1550,11 +1551,11 @@
       <c r="V9" s="3"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A10" s="39"/>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="42"/>
-      <c r="E10" s="33"/>
+      <c r="A10" s="36"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="41"/>
       <c r="F10" s="9" t="s">
         <v>21</v>
       </c>
@@ -1568,14 +1569,14 @@
         <v>22</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>23</v>
+        <v>76</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="L10" s="33"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="32"/>
+        <v>40</v>
+      </c>
+      <c r="L10" s="41"/>
+      <c r="M10" s="44"/>
+      <c r="N10" s="40"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
@@ -1586,41 +1587,41 @@
       <c r="V10" s="3"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A11" s="39"/>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
+      <c r="A11" s="36"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="36"/>
       <c r="D11" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="G11" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="H11" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="I11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="J11" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="K11" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="J11" s="13" t="s">
+      <c r="L11" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="M11" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="L11" s="13" t="s">
+      <c r="N11" s="13" t="s">
         <v>33</v>
-      </c>
-      <c r="M11" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="N11" s="13" t="s">
-        <v>35</v>
       </c>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1632,22 +1633,22 @@
       <c r="V11" s="3"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A12" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
-      <c r="K12" s="28"/>
-      <c r="L12" s="28"/>
-      <c r="M12" s="28"/>
-      <c r="N12" s="28"/>
+      <c r="A12" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="46"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="46"/>
+      <c r="I12" s="46"/>
+      <c r="J12" s="46"/>
+      <c r="K12" s="46"/>
+      <c r="L12" s="46"/>
+      <c r="M12" s="46"/>
+      <c r="N12" s="46"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
@@ -1662,36 +1663,36 @@
       <c r="A13" s="24">
         <v>1</v>
       </c>
-      <c r="B13" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="50">
+      <c r="B13" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="47"/>
+      <c r="D13" s="27">
         <f>SUM(E13:L13)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="47">
-        <v>0</v>
-      </c>
-      <c r="F13" s="47">
-        <v>0</v>
-      </c>
-      <c r="G13" s="47">
-        <v>0</v>
-      </c>
-      <c r="H13" s="47">
-        <v>0</v>
-      </c>
-      <c r="I13" s="47">
-        <v>0</v>
-      </c>
-      <c r="J13" s="47">
-        <v>0</v>
-      </c>
-      <c r="K13" s="47">
-        <v>0</v>
-      </c>
-      <c r="L13" s="47">
+      <c r="E13" s="25">
+        <v>0</v>
+      </c>
+      <c r="F13" s="25">
+        <v>0</v>
+      </c>
+      <c r="G13" s="25">
+        <v>0</v>
+      </c>
+      <c r="H13" s="25">
+        <v>0</v>
+      </c>
+      <c r="I13" s="25">
+        <v>0</v>
+      </c>
+      <c r="J13" s="25">
+        <v>0</v>
+      </c>
+      <c r="K13" s="25">
+        <v>0</v>
+      </c>
+      <c r="L13" s="25">
         <v>0</v>
       </c>
       <c r="M13" s="24"/>
@@ -1709,36 +1710,36 @@
       <c r="A14" s="24">
         <v>2</v>
       </c>
-      <c r="B14" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="50">
+      <c r="B14" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="47"/>
+      <c r="D14" s="27">
         <f>SUM(E14:L14)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="47">
-        <v>0</v>
-      </c>
-      <c r="F14" s="47">
-        <v>0</v>
-      </c>
-      <c r="G14" s="47">
-        <v>0</v>
-      </c>
-      <c r="H14" s="47">
-        <v>0</v>
-      </c>
-      <c r="I14" s="47">
-        <v>0</v>
-      </c>
-      <c r="J14" s="47">
-        <v>0</v>
-      </c>
-      <c r="K14" s="47">
-        <v>0</v>
-      </c>
-      <c r="L14" s="47">
+      <c r="E14" s="25">
+        <v>0</v>
+      </c>
+      <c r="F14" s="25">
+        <v>0</v>
+      </c>
+      <c r="G14" s="25">
+        <v>0</v>
+      </c>
+      <c r="H14" s="25">
+        <v>0</v>
+      </c>
+      <c r="I14" s="25">
+        <v>0</v>
+      </c>
+      <c r="J14" s="25">
+        <v>0</v>
+      </c>
+      <c r="K14" s="25">
+        <v>0</v>
+      </c>
+      <c r="L14" s="25">
         <v>0</v>
       </c>
       <c r="M14" s="24"/>
@@ -1756,36 +1757,36 @@
       <c r="A15" s="24">
         <v>3</v>
       </c>
-      <c r="B15" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="29"/>
-      <c r="D15" s="50">
+      <c r="B15" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="47"/>
+      <c r="D15" s="27">
         <f>SUM(E15:L15)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="47">
-        <v>0</v>
-      </c>
-      <c r="F15" s="47">
-        <v>0</v>
-      </c>
-      <c r="G15" s="47">
-        <v>0</v>
-      </c>
-      <c r="H15" s="47">
-        <v>0</v>
-      </c>
-      <c r="I15" s="47">
-        <v>0</v>
-      </c>
-      <c r="J15" s="47">
-        <v>0</v>
-      </c>
-      <c r="K15" s="47">
-        <v>0</v>
-      </c>
-      <c r="L15" s="47">
+      <c r="E15" s="25">
+        <v>0</v>
+      </c>
+      <c r="F15" s="25">
+        <v>0</v>
+      </c>
+      <c r="G15" s="25">
+        <v>0</v>
+      </c>
+      <c r="H15" s="25">
+        <v>0</v>
+      </c>
+      <c r="I15" s="25">
+        <v>0</v>
+      </c>
+      <c r="J15" s="25">
+        <v>0</v>
+      </c>
+      <c r="K15" s="25">
+        <v>0</v>
+      </c>
+      <c r="L15" s="25">
         <v>0</v>
       </c>
       <c r="M15" s="14"/>
@@ -1800,41 +1801,41 @@
       <c r="V15" s="3"/>
     </row>
     <row r="16" spans="1:24" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="30">
+      <c r="A16" s="48">
         <v>4</v>
       </c>
-      <c r="B16" s="31" t="s">
-        <v>40</v>
+      <c r="B16" s="49" t="s">
+        <v>38</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="D16" s="50">
+        <v>39</v>
+      </c>
+      <c r="D16" s="27">
         <f>SUM(E16:L16)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="47">
-        <v>0</v>
-      </c>
-      <c r="F16" s="47">
-        <v>0</v>
-      </c>
-      <c r="G16" s="47">
-        <v>0</v>
-      </c>
-      <c r="H16" s="47">
-        <v>0</v>
-      </c>
-      <c r="I16" s="47">
-        <v>0</v>
-      </c>
-      <c r="J16" s="47">
-        <v>0</v>
-      </c>
-      <c r="K16" s="47">
-        <v>0</v>
-      </c>
-      <c r="L16" s="47">
+      <c r="E16" s="25">
+        <v>0</v>
+      </c>
+      <c r="F16" s="25">
+        <v>0</v>
+      </c>
+      <c r="G16" s="25">
+        <v>0</v>
+      </c>
+      <c r="H16" s="25">
+        <v>0</v>
+      </c>
+      <c r="I16" s="25">
+        <v>0</v>
+      </c>
+      <c r="J16" s="25">
+        <v>0</v>
+      </c>
+      <c r="K16" s="25">
+        <v>0</v>
+      </c>
+      <c r="L16" s="25">
         <v>0</v>
       </c>
       <c r="M16" s="14"/>
@@ -1849,37 +1850,37 @@
       <c r="V16" s="3"/>
     </row>
     <row r="17" spans="1:22" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="30"/>
-      <c r="B17" s="31"/>
+      <c r="A17" s="48"/>
+      <c r="B17" s="49"/>
       <c r="C17" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="50">
+        <v>40</v>
+      </c>
+      <c r="D17" s="27">
         <f>SUM(E17:L17)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="47">
-        <v>0</v>
-      </c>
-      <c r="F17" s="47">
-        <v>0</v>
-      </c>
-      <c r="G17" s="47">
-        <v>0</v>
-      </c>
-      <c r="H17" s="47">
-        <v>0</v>
-      </c>
-      <c r="I17" s="47">
-        <v>0</v>
-      </c>
-      <c r="J17" s="47">
-        <v>0</v>
-      </c>
-      <c r="K17" s="47">
-        <v>0</v>
-      </c>
-      <c r="L17" s="47">
+      <c r="E17" s="25">
+        <v>0</v>
+      </c>
+      <c r="F17" s="25">
+        <v>0</v>
+      </c>
+      <c r="G17" s="25">
+        <v>0</v>
+      </c>
+      <c r="H17" s="25">
+        <v>0</v>
+      </c>
+      <c r="I17" s="25">
+        <v>0</v>
+      </c>
+      <c r="J17" s="25">
+        <v>0</v>
+      </c>
+      <c r="K17" s="25">
+        <v>0</v>
+      </c>
+      <c r="L17" s="25">
         <v>0</v>
       </c>
       <c r="M17" s="14"/>
@@ -1894,44 +1895,44 @@
       <c r="V17" s="3"/>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A18" s="52" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="48">
+      <c r="A18" s="50" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" s="50"/>
+      <c r="C18" s="50"/>
+      <c r="D18" s="26">
         <f>SUM(D13:D17)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="48">
+      <c r="E18" s="26">
         <f>SUM(E13:E17)</f>
         <v>0</v>
       </c>
-      <c r="F18" s="48">
+      <c r="F18" s="26">
         <f t="shared" ref="F18:L18" si="0">SUM(F13:F17)</f>
         <v>0</v>
       </c>
-      <c r="G18" s="48">
+      <c r="G18" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="48">
+      <c r="H18" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I18" s="48">
+      <c r="I18" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J18" s="48">
+      <c r="J18" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K18" s="48">
+      <c r="K18" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L18" s="48">
+      <c r="L18" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1947,22 +1948,22 @@
       <c r="V18" s="3"/>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A19" s="53" t="s">
-        <v>44</v>
-      </c>
-      <c r="B19" s="53"/>
-      <c r="C19" s="53"/>
-      <c r="D19" s="53"/>
-      <c r="E19" s="53"/>
-      <c r="F19" s="53"/>
-      <c r="G19" s="53"/>
-      <c r="H19" s="53"/>
-      <c r="I19" s="53"/>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="L19" s="53"/>
-      <c r="M19" s="53"/>
-      <c r="N19" s="53"/>
+      <c r="A19" s="51" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="51"/>
+      <c r="C19" s="51"/>
+      <c r="D19" s="51"/>
+      <c r="E19" s="51"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="51"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="51"/>
+      <c r="K19" s="51"/>
+      <c r="L19" s="51"/>
+      <c r="M19" s="51"/>
+      <c r="N19" s="51"/>
       <c r="O19" s="3"/>
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
@@ -1974,38 +1975,38 @@
     </row>
     <row r="20" spans="1:22" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="B20" s="54" t="s">
-        <v>46</v>
-      </c>
-      <c r="C20" s="54"/>
-      <c r="D20" s="50">
+        <v>43</v>
+      </c>
+      <c r="B20" s="45" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="45"/>
+      <c r="D20" s="27">
         <f>SUM(E20:L20)</f>
         <v>0</v>
       </c>
-      <c r="E20" s="47">
-        <v>0</v>
-      </c>
-      <c r="F20" s="47">
-        <v>0</v>
-      </c>
-      <c r="G20" s="47">
-        <v>0</v>
-      </c>
-      <c r="H20" s="47">
-        <v>0</v>
-      </c>
-      <c r="I20" s="47">
-        <v>0</v>
-      </c>
-      <c r="J20" s="47">
-        <v>0</v>
-      </c>
-      <c r="K20" s="47">
-        <v>0</v>
-      </c>
-      <c r="L20" s="47">
+      <c r="E20" s="25">
+        <v>0</v>
+      </c>
+      <c r="F20" s="25">
+        <v>0</v>
+      </c>
+      <c r="G20" s="25">
+        <v>0</v>
+      </c>
+      <c r="H20" s="25">
+        <v>0</v>
+      </c>
+      <c r="I20" s="25">
+        <v>0</v>
+      </c>
+      <c r="J20" s="25">
+        <v>0</v>
+      </c>
+      <c r="K20" s="25">
+        <v>0</v>
+      </c>
+      <c r="L20" s="25">
         <v>0</v>
       </c>
       <c r="M20" s="14"/>
@@ -2021,38 +2022,38 @@
     </row>
     <row r="21" spans="1:22" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B21" s="54" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" s="54"/>
-      <c r="D21" s="50">
+        <v>45</v>
+      </c>
+      <c r="B21" s="45" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="45"/>
+      <c r="D21" s="27">
         <f>SUM(E21:L21)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="47">
-        <v>0</v>
-      </c>
-      <c r="F21" s="47">
-        <v>0</v>
-      </c>
-      <c r="G21" s="47">
-        <v>0</v>
-      </c>
-      <c r="H21" s="47">
-        <v>0</v>
-      </c>
-      <c r="I21" s="47">
-        <v>0</v>
-      </c>
-      <c r="J21" s="47">
-        <v>0</v>
-      </c>
-      <c r="K21" s="47">
-        <v>0</v>
-      </c>
-      <c r="L21" s="47">
+      <c r="E21" s="25">
+        <v>0</v>
+      </c>
+      <c r="F21" s="25">
+        <v>0</v>
+      </c>
+      <c r="G21" s="25">
+        <v>0</v>
+      </c>
+      <c r="H21" s="25">
+        <v>0</v>
+      </c>
+      <c r="I21" s="25">
+        <v>0</v>
+      </c>
+      <c r="J21" s="25">
+        <v>0</v>
+      </c>
+      <c r="K21" s="25">
+        <v>0</v>
+      </c>
+      <c r="L21" s="25">
         <v>0</v>
       </c>
       <c r="M21" s="14"/>
@@ -2068,38 +2069,38 @@
     </row>
     <row r="22" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" s="54" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="54"/>
-      <c r="D22" s="50">
+        <v>47</v>
+      </c>
+      <c r="B22" s="45" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="45"/>
+      <c r="D22" s="27">
         <f>SUM(E22:L22)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="47">
-        <v>0</v>
-      </c>
-      <c r="F22" s="47">
-        <v>0</v>
-      </c>
-      <c r="G22" s="47">
-        <v>0</v>
-      </c>
-      <c r="H22" s="47">
-        <v>0</v>
-      </c>
-      <c r="I22" s="47">
-        <v>0</v>
-      </c>
-      <c r="J22" s="47">
-        <v>0</v>
-      </c>
-      <c r="K22" s="47">
-        <v>0</v>
-      </c>
-      <c r="L22" s="47">
+      <c r="E22" s="25">
+        <v>0</v>
+      </c>
+      <c r="F22" s="25">
+        <v>0</v>
+      </c>
+      <c r="G22" s="25">
+        <v>0</v>
+      </c>
+      <c r="H22" s="25">
+        <v>0</v>
+      </c>
+      <c r="I22" s="25">
+        <v>0</v>
+      </c>
+      <c r="J22" s="25">
+        <v>0</v>
+      </c>
+      <c r="K22" s="25">
+        <v>0</v>
+      </c>
+      <c r="L22" s="25">
         <v>0</v>
       </c>
       <c r="M22" s="14"/>
@@ -2115,38 +2116,38 @@
     </row>
     <row r="23" spans="1:22" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23" s="54" t="s">
-        <v>52</v>
-      </c>
-      <c r="C23" s="54"/>
-      <c r="D23" s="50">
+        <v>49</v>
+      </c>
+      <c r="B23" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="45"/>
+      <c r="D23" s="27">
         <f>SUM(E23:L23)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="47">
-        <v>0</v>
-      </c>
-      <c r="F23" s="47">
-        <v>0</v>
-      </c>
-      <c r="G23" s="47">
-        <v>0</v>
-      </c>
-      <c r="H23" s="47">
-        <v>0</v>
-      </c>
-      <c r="I23" s="47">
-        <v>0</v>
-      </c>
-      <c r="J23" s="47">
-        <v>0</v>
-      </c>
-      <c r="K23" s="47">
-        <v>0</v>
-      </c>
-      <c r="L23" s="47">
+      <c r="E23" s="25">
+        <v>0</v>
+      </c>
+      <c r="F23" s="25">
+        <v>0</v>
+      </c>
+      <c r="G23" s="25">
+        <v>0</v>
+      </c>
+      <c r="H23" s="25">
+        <v>0</v>
+      </c>
+      <c r="I23" s="25">
+        <v>0</v>
+      </c>
+      <c r="J23" s="25">
+        <v>0</v>
+      </c>
+      <c r="K23" s="25">
+        <v>0</v>
+      </c>
+      <c r="L23" s="25">
         <v>0</v>
       </c>
       <c r="M23" s="14"/>
@@ -2162,38 +2163,38 @@
     </row>
     <row r="24" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="54" t="s">
-        <v>54</v>
-      </c>
-      <c r="C24" s="54"/>
-      <c r="D24" s="50">
+        <v>51</v>
+      </c>
+      <c r="B24" s="45" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="45"/>
+      <c r="D24" s="27">
         <f>SUM(E24:L24)</f>
         <v>0</v>
       </c>
-      <c r="E24" s="47">
-        <v>0</v>
-      </c>
-      <c r="F24" s="47">
-        <v>0</v>
-      </c>
-      <c r="G24" s="47">
-        <v>0</v>
-      </c>
-      <c r="H24" s="47">
-        <v>0</v>
-      </c>
-      <c r="I24" s="47">
-        <v>0</v>
-      </c>
-      <c r="J24" s="47">
-        <v>0</v>
-      </c>
-      <c r="K24" s="47">
-        <v>0</v>
-      </c>
-      <c r="L24" s="47">
+      <c r="E24" s="25">
+        <v>0</v>
+      </c>
+      <c r="F24" s="25">
+        <v>0</v>
+      </c>
+      <c r="G24" s="25">
+        <v>0</v>
+      </c>
+      <c r="H24" s="25">
+        <v>0</v>
+      </c>
+      <c r="I24" s="25">
+        <v>0</v>
+      </c>
+      <c r="J24" s="25">
+        <v>0</v>
+      </c>
+      <c r="K24" s="25">
+        <v>0</v>
+      </c>
+      <c r="L24" s="25">
         <v>0</v>
       </c>
       <c r="M24" s="14"/>
@@ -2209,38 +2210,38 @@
     </row>
     <row r="25" spans="1:22" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" s="54" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25" s="54"/>
-      <c r="D25" s="50">
+        <v>53</v>
+      </c>
+      <c r="B25" s="45" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="45"/>
+      <c r="D25" s="27">
         <f>SUM(E25:L25)</f>
         <v>0</v>
       </c>
-      <c r="E25" s="47">
-        <v>0</v>
-      </c>
-      <c r="F25" s="47">
-        <v>0</v>
-      </c>
-      <c r="G25" s="47">
-        <v>0</v>
-      </c>
-      <c r="H25" s="47">
-        <v>0</v>
-      </c>
-      <c r="I25" s="47">
-        <v>0</v>
-      </c>
-      <c r="J25" s="47">
-        <v>0</v>
-      </c>
-      <c r="K25" s="47">
-        <v>0</v>
-      </c>
-      <c r="L25" s="47">
+      <c r="E25" s="25">
+        <v>0</v>
+      </c>
+      <c r="F25" s="25">
+        <v>0</v>
+      </c>
+      <c r="G25" s="25">
+        <v>0</v>
+      </c>
+      <c r="H25" s="25">
+        <v>0</v>
+      </c>
+      <c r="I25" s="25">
+        <v>0</v>
+      </c>
+      <c r="J25" s="25">
+        <v>0</v>
+      </c>
+      <c r="K25" s="25">
+        <v>0</v>
+      </c>
+      <c r="L25" s="25">
         <v>0</v>
       </c>
       <c r="M25" s="14"/>
@@ -2256,38 +2257,38 @@
     </row>
     <row r="26" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="54" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" s="54"/>
-      <c r="D26" s="50">
+        <v>55</v>
+      </c>
+      <c r="B26" s="45" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="45"/>
+      <c r="D26" s="27">
         <f>SUM(E26:L26)</f>
         <v>0</v>
       </c>
-      <c r="E26" s="47">
-        <v>0</v>
-      </c>
-      <c r="F26" s="47">
-        <v>0</v>
-      </c>
-      <c r="G26" s="47">
-        <v>0</v>
-      </c>
-      <c r="H26" s="47">
-        <v>0</v>
-      </c>
-      <c r="I26" s="47">
-        <v>0</v>
-      </c>
-      <c r="J26" s="47">
-        <v>0</v>
-      </c>
-      <c r="K26" s="47">
-        <v>0</v>
-      </c>
-      <c r="L26" s="47">
+      <c r="E26" s="25">
+        <v>0</v>
+      </c>
+      <c r="F26" s="25">
+        <v>0</v>
+      </c>
+      <c r="G26" s="25">
+        <v>0</v>
+      </c>
+      <c r="H26" s="25">
+        <v>0</v>
+      </c>
+      <c r="I26" s="25">
+        <v>0</v>
+      </c>
+      <c r="J26" s="25">
+        <v>0</v>
+      </c>
+      <c r="K26" s="25">
+        <v>0</v>
+      </c>
+      <c r="L26" s="25">
         <v>0</v>
       </c>
       <c r="M26" s="14"/>
@@ -2303,38 +2304,38 @@
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A27" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="B27" s="55" t="s">
-        <v>60</v>
-      </c>
-      <c r="C27" s="54"/>
-      <c r="D27" s="50">
+        <v>57</v>
+      </c>
+      <c r="B27" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" s="45"/>
+      <c r="D27" s="27">
         <f>SUM(E27:L27)</f>
         <v>0</v>
       </c>
-      <c r="E27" s="47">
-        <v>0</v>
-      </c>
-      <c r="F27" s="47">
-        <v>0</v>
-      </c>
-      <c r="G27" s="47">
-        <v>0</v>
-      </c>
-      <c r="H27" s="47">
-        <v>0</v>
-      </c>
-      <c r="I27" s="47">
-        <v>0</v>
-      </c>
-      <c r="J27" s="47">
-        <v>0</v>
-      </c>
-      <c r="K27" s="47">
-        <v>0</v>
-      </c>
-      <c r="L27" s="47">
+      <c r="E27" s="25">
+        <v>0</v>
+      </c>
+      <c r="F27" s="25">
+        <v>0</v>
+      </c>
+      <c r="G27" s="25">
+        <v>0</v>
+      </c>
+      <c r="H27" s="25">
+        <v>0</v>
+      </c>
+      <c r="I27" s="25">
+        <v>0</v>
+      </c>
+      <c r="J27" s="25">
+        <v>0</v>
+      </c>
+      <c r="K27" s="25">
+        <v>0</v>
+      </c>
+      <c r="L27" s="25">
         <v>0</v>
       </c>
       <c r="M27" s="14"/>
@@ -2350,40 +2351,40 @@
     </row>
     <row r="28" spans="1:22" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="18"/>
-      <c r="B28" s="51" t="s">
-        <v>61</v>
-      </c>
-      <c r="C28" s="51"/>
-      <c r="D28" s="50">
+      <c r="B28" s="54" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="54"/>
+      <c r="D28" s="27">
         <f>SUM(E28:L28)</f>
         <v>0</v>
       </c>
-      <c r="E28" s="47">
-        <v>0</v>
-      </c>
-      <c r="F28" s="47">
-        <v>0</v>
-      </c>
-      <c r="G28" s="47">
-        <v>0</v>
-      </c>
-      <c r="H28" s="47">
-        <v>0</v>
-      </c>
-      <c r="I28" s="47">
-        <v>0</v>
-      </c>
-      <c r="J28" s="47">
-        <v>0</v>
-      </c>
-      <c r="K28" s="47">
-        <v>0</v>
-      </c>
-      <c r="L28" s="47">
-        <v>0</v>
-      </c>
-      <c r="M28" s="14"/>
-      <c r="N28" s="24"/>
+      <c r="E28" s="25">
+        <v>0</v>
+      </c>
+      <c r="F28" s="25">
+        <v>0</v>
+      </c>
+      <c r="G28" s="25">
+        <v>0</v>
+      </c>
+      <c r="H28" s="25">
+        <v>0</v>
+      </c>
+      <c r="I28" s="25">
+        <v>0</v>
+      </c>
+      <c r="J28" s="25">
+        <v>0</v>
+      </c>
+      <c r="K28" s="25">
+        <v>0</v>
+      </c>
+      <c r="L28" s="25">
+        <v>0</v>
+      </c>
+      <c r="M28" s="60"/>
+      <c r="N28" s="60"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
@@ -2395,40 +2396,40 @@
     </row>
     <row r="29" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="18"/>
-      <c r="B29" s="51" t="s">
-        <v>62</v>
-      </c>
-      <c r="C29" s="51"/>
-      <c r="D29" s="50">
+      <c r="B29" s="54" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" s="54"/>
+      <c r="D29" s="27">
         <f>SUM(E29:L29)</f>
         <v>0</v>
       </c>
-      <c r="E29" s="47">
-        <v>0</v>
-      </c>
-      <c r="F29" s="47">
-        <v>0</v>
-      </c>
-      <c r="G29" s="47">
-        <v>0</v>
-      </c>
-      <c r="H29" s="47">
-        <v>0</v>
-      </c>
-      <c r="I29" s="47">
-        <v>0</v>
-      </c>
-      <c r="J29" s="47">
-        <v>0</v>
-      </c>
-      <c r="K29" s="47">
-        <v>0</v>
-      </c>
-      <c r="L29" s="47">
-        <v>0</v>
-      </c>
-      <c r="M29" s="14"/>
-      <c r="N29" s="24"/>
+      <c r="E29" s="25">
+        <v>0</v>
+      </c>
+      <c r="F29" s="25">
+        <v>0</v>
+      </c>
+      <c r="G29" s="25">
+        <v>0</v>
+      </c>
+      <c r="H29" s="25">
+        <v>0</v>
+      </c>
+      <c r="I29" s="25">
+        <v>0</v>
+      </c>
+      <c r="J29" s="25">
+        <v>0</v>
+      </c>
+      <c r="K29" s="25">
+        <v>0</v>
+      </c>
+      <c r="L29" s="25">
+        <v>0</v>
+      </c>
+      <c r="M29" s="60"/>
+      <c r="N29" s="60"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
@@ -2439,44 +2440,44 @@
       <c r="V29" s="3"/>
     </row>
     <row r="30" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="56" t="s">
-        <v>63</v>
-      </c>
-      <c r="B30" s="56"/>
-      <c r="C30" s="56"/>
-      <c r="D30" s="50">
+      <c r="A30" s="55" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="55"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="27">
         <f>SUM(E30:L30)</f>
         <v>0</v>
       </c>
-      <c r="E30" s="48">
+      <c r="E30" s="26">
         <f>SUM(E20:E29)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="48">
+      <c r="F30" s="26">
         <f>SUM(F20:F29)</f>
         <v>0</v>
       </c>
-      <c r="G30" s="48">
+      <c r="G30" s="26">
         <f>SUM(G20:G29)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="48">
+      <c r="H30" s="26">
         <f>SUM(H20:H29)</f>
         <v>0</v>
       </c>
-      <c r="I30" s="48">
+      <c r="I30" s="26">
         <f>SUM(I20:I29)</f>
         <v>0</v>
       </c>
-      <c r="J30" s="48">
+      <c r="J30" s="26">
         <f>SUM(J20:J29)</f>
         <v>0</v>
       </c>
-      <c r="K30" s="48">
+      <c r="K30" s="26">
         <f>SUM(K20:K29)</f>
         <v>0</v>
       </c>
-      <c r="L30" s="48">
+      <c r="L30" s="26">
         <f>SUM(L20:L29)</f>
         <v>0</v>
       </c>
@@ -2492,37 +2493,37 @@
       <c r="V30" s="3"/>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A31" s="49" t="s">
-        <v>64</v>
-      </c>
-      <c r="B31" s="49"/>
-      <c r="C31" s="49"/>
-      <c r="D31" s="50">
+      <c r="A31" s="59" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" s="59"/>
+      <c r="C31" s="59"/>
+      <c r="D31" s="27">
         <f>SUM(E31:L31)</f>
         <v>0</v>
       </c>
-      <c r="E31" s="47">
-        <v>0</v>
-      </c>
-      <c r="F31" s="47">
-        <v>0</v>
-      </c>
-      <c r="G31" s="47">
-        <v>0</v>
-      </c>
-      <c r="H31" s="47">
-        <v>0</v>
-      </c>
-      <c r="I31" s="47">
-        <v>0</v>
-      </c>
-      <c r="J31" s="47">
-        <v>0</v>
-      </c>
-      <c r="K31" s="47">
-        <v>0</v>
-      </c>
-      <c r="L31" s="47">
+      <c r="E31" s="25">
+        <v>0</v>
+      </c>
+      <c r="F31" s="25">
+        <v>0</v>
+      </c>
+      <c r="G31" s="25">
+        <v>0</v>
+      </c>
+      <c r="H31" s="25">
+        <v>0</v>
+      </c>
+      <c r="I31" s="25">
+        <v>0</v>
+      </c>
+      <c r="J31" s="25">
+        <v>0</v>
+      </c>
+      <c r="K31" s="25">
+        <v>0</v>
+      </c>
+      <c r="L31" s="25">
         <v>0</v>
       </c>
       <c r="M31" s="14"/>
@@ -2537,44 +2538,44 @@
       <c r="V31" s="3"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A32" s="57" t="s">
-        <v>65</v>
-      </c>
-      <c r="B32" s="57"/>
-      <c r="C32" s="57"/>
-      <c r="D32" s="48">
+      <c r="A32" s="56" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="56"/>
+      <c r="C32" s="56"/>
+      <c r="D32" s="26">
         <f>D18+D30+D31</f>
         <v>0</v>
       </c>
-      <c r="E32" s="48">
+      <c r="E32" s="26">
         <f>E18+E30+E31</f>
         <v>0</v>
       </c>
-      <c r="F32" s="48">
+      <c r="F32" s="26">
         <f>F18+F30+F31</f>
         <v>0</v>
       </c>
-      <c r="G32" s="48">
+      <c r="G32" s="26">
         <f>G18+G30+G31</f>
         <v>0</v>
       </c>
-      <c r="H32" s="48">
+      <c r="H32" s="26">
         <f>H18+H30+H31</f>
         <v>0</v>
       </c>
-      <c r="I32" s="48">
+      <c r="I32" s="26">
         <f>I18+I30+I31</f>
         <v>0</v>
       </c>
-      <c r="J32" s="48">
+      <c r="J32" s="26">
         <f>J18+J30+J31</f>
         <v>0</v>
       </c>
-      <c r="K32" s="48">
+      <c r="K32" s="26">
         <f>K18+K30+K31</f>
         <v>0</v>
       </c>
-      <c r="L32" s="48">
+      <c r="L32" s="26">
         <f>L18+L30+L31</f>
         <v>0</v>
       </c>
@@ -2599,13 +2600,13 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="K33" s="26"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="26"/>
-      <c r="N33" s="26"/>
+      <c r="J33" s="57" t="s">
+        <v>64</v>
+      </c>
+      <c r="K33" s="57"/>
+      <c r="L33" s="57"/>
+      <c r="M33" s="57"/>
+      <c r="N33" s="57"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
@@ -2617,23 +2618,23 @@
     </row>
     <row r="34" spans="1:22" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A34" s="3"/>
-      <c r="B34" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="C34" s="27"/>
+      <c r="B34" s="58" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="58"/>
       <c r="D34" s="22"/>
       <c r="E34" s="22"/>
       <c r="F34" s="22"/>
       <c r="G34" s="22"/>
       <c r="H34" s="22"/>
       <c r="I34" s="22"/>
-      <c r="J34" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="K34" s="27"/>
-      <c r="L34" s="27"/>
-      <c r="M34" s="27"/>
-      <c r="N34" s="27"/>
+      <c r="J34" s="58" t="s">
+        <v>66</v>
+      </c>
+      <c r="K34" s="58"/>
+      <c r="L34" s="58"/>
+      <c r="M34" s="58"/>
+      <c r="N34" s="58"/>
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
@@ -2645,23 +2646,23 @@
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
-      <c r="B35" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="C35" s="25"/>
+      <c r="B35" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" s="52"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
-      <c r="J35" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="K35" s="25"/>
-      <c r="L35" s="25"/>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
+      <c r="J35" s="52" t="s">
+        <v>68</v>
+      </c>
+      <c r="K35" s="52"/>
+      <c r="L35" s="52"/>
+      <c r="M35" s="52"/>
+      <c r="N35" s="52"/>
       <c r="O35" s="3"/>
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
@@ -2673,40 +2674,6 @@
     </row>
   </sheetData>
   <mergeCells count="48">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="G5:N5"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="A8:C11"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:L8"/>
-    <mergeCell ref="N8:N10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:N19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="J35:N35"/>
     <mergeCell ref="B24:C24"/>
@@ -2721,6 +2688,40 @@
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="J34:N34"/>
     <mergeCell ref="A31:C31"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:N19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="A8:C11"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:L8"/>
+    <mergeCell ref="N8:N10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="G5:N5"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
- Added VI translations for reports - Added Active Screening counting to Patients Report - Removed AFB fields from Patients Report - Added TB4 counting to Patients Report
</commit_message>
<xml_diff>
--- a/api/templates/xpert_m4b1_patients/en.xlsx
+++ b/api/templates/xpert_m4b1_patients/en.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\xpert_m4b1_patients\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0853380D-4218-4CF2-8012-16534167D580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB16FAB-483A-46D1-B0FA-6A4E320430C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B124328-57BC-4FCF-919D-A7394F83025A}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="75">
   <si>
     <t xml:space="preserve">MINISTRY OF HEALTH </t>
   </si>
@@ -216,12 +216,6 @@
   </si>
   <si>
     <t>New TB patients</t>
-  </si>
-  <si>
-    <t>A8a.Pulmonary TB patients AFB(+)</t>
-  </si>
-  <si>
-    <t>A8b.Pulmonary TB patients AFB(-)</t>
   </si>
   <si>
     <t>Total number of groups diagnosed with MDR TB  (II)</t>
@@ -276,7 +270,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,12 +375,6 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="163"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -508,7 +496,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -579,7 +567,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -702,7 +690,7 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -710,10 +698,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
@@ -722,20 +706,16 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -782,7 +762,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>1276350</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>168275</xdr:rowOff>
+          <xdr:rowOff>161925</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -849,7 +829,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>114300</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>168275</xdr:rowOff>
+          <xdr:rowOff>161925</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -914,9 +894,9 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>644525</xdr:colOff>
+          <xdr:colOff>638175</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>168275</xdr:rowOff>
+          <xdr:rowOff>161925</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1270,7 +1250,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDC72112-4D5E-4A55-BF7D-4A69BC3E2ED4}">
-  <dimension ref="A1:X35"/>
+  <dimension ref="A1:X33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
@@ -1360,7 +1340,7 @@
     </row>
     <row r="4" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B4" s="32"/>
       <c r="C4" s="32"/>
@@ -1390,7 +1370,7 @@
       </c>
       <c r="B5" s="33"/>
       <c r="C5" s="33" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D5" s="33"/>
       <c r="E5" s="33"/>
@@ -1398,7 +1378,7 @@
         <v>5</v>
       </c>
       <c r="G5" s="34" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H5" s="34"/>
       <c r="I5" s="34"/>
@@ -1422,7 +1402,7 @@
       </c>
       <c r="B6" s="28"/>
       <c r="C6" s="33" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D6" s="33"/>
       <c r="E6" s="33"/>
@@ -1430,7 +1410,7 @@
         <v>7</v>
       </c>
       <c r="G6" s="34" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="H6" s="34"/>
       <c r="I6" s="34"/>
@@ -1438,7 +1418,7 @@
         <v>8</v>
       </c>
       <c r="K6" s="34" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L6" s="34"/>
       <c r="M6" s="34"/>
@@ -1537,7 +1517,7 @@
       </c>
       <c r="K9" s="41"/>
       <c r="L9" s="41" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="M9" s="43"/>
       <c r="N9" s="40"/>
@@ -1569,7 +1549,7 @@
         <v>22</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>40</v>
@@ -1936,7 +1916,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M18" s="16"/>
+      <c r="M18" s="16">
+        <f>SUM(M13:M17)</f>
+        <v>0</v>
+      </c>
       <c r="N18" s="17"/>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
@@ -1982,7 +1965,7 @@
       </c>
       <c r="C20" s="45"/>
       <c r="D20" s="27">
-        <f>SUM(E20:L20)</f>
+        <f t="shared" ref="D20:D27" si="1">SUM(E20:L20)</f>
         <v>0</v>
       </c>
       <c r="E20" s="25">
@@ -2029,7 +2012,7 @@
       </c>
       <c r="C21" s="45"/>
       <c r="D21" s="27">
-        <f>SUM(E21:L21)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E21" s="25">
@@ -2076,7 +2059,7 @@
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="27">
-        <f>SUM(E22:L22)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E22" s="25">
@@ -2123,7 +2106,7 @@
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="27">
-        <f>SUM(E23:L23)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E23" s="25">
@@ -2170,7 +2153,7 @@
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="27">
-        <f>SUM(E24:L24)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E24" s="25">
@@ -2217,7 +2200,7 @@
       </c>
       <c r="C25" s="45"/>
       <c r="D25" s="27">
-        <f>SUM(E25:L25)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E25" s="25">
@@ -2264,7 +2247,7 @@
       </c>
       <c r="C26" s="45"/>
       <c r="D26" s="27">
-        <f>SUM(E26:L26)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E26" s="25">
@@ -2311,7 +2294,7 @@
       </c>
       <c r="C27" s="45"/>
       <c r="D27" s="27">
-        <f>SUM(E27:L27)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E27" s="25">
@@ -2349,42 +2332,53 @@
       <c r="U27" s="3"/>
       <c r="V27" s="3"/>
     </row>
-    <row r="28" spans="1:22" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="18"/>
-      <c r="B28" s="54" t="s">
+    <row r="28" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="54" t="s">
         <v>59</v>
       </c>
+      <c r="B28" s="54"/>
       <c r="C28" s="54"/>
       <c r="D28" s="27">
         <f>SUM(E28:L28)</f>
         <v>0</v>
       </c>
-      <c r="E28" s="25">
-        <v>0</v>
-      </c>
-      <c r="F28" s="25">
-        <v>0</v>
-      </c>
-      <c r="G28" s="25">
-        <v>0</v>
-      </c>
-      <c r="H28" s="25">
-        <v>0</v>
-      </c>
-      <c r="I28" s="25">
-        <v>0</v>
-      </c>
-      <c r="J28" s="25">
-        <v>0</v>
-      </c>
-      <c r="K28" s="25">
-        <v>0</v>
-      </c>
-      <c r="L28" s="25">
-        <v>0</v>
-      </c>
-      <c r="M28" s="60"/>
-      <c r="N28" s="60"/>
+      <c r="E28" s="26">
+        <f t="shared" ref="E28:L28" si="2">SUM(E20:E27)</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G28" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H28" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I28" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J28" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K28" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L28" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M28" s="16">
+        <f>SUM(M20:M27)</f>
+        <v>0</v>
+      </c>
+      <c r="N28" s="20"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
@@ -2394,12 +2388,12 @@
       <c r="U28" s="3"/>
       <c r="V28" s="3"/>
     </row>
-    <row r="29" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="18"/>
-      <c r="B29" s="54" t="s">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A29" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="54"/>
+      <c r="B29" s="58"/>
+      <c r="C29" s="58"/>
       <c r="D29" s="27">
         <f>SUM(E29:L29)</f>
         <v>0</v>
@@ -2428,8 +2422,8 @@
       <c r="L29" s="25">
         <v>0</v>
       </c>
-      <c r="M29" s="60"/>
-      <c r="N29" s="60"/>
+      <c r="M29" s="14"/>
+      <c r="N29" s="24"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
@@ -2439,50 +2433,53 @@
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
     </row>
-    <row r="30" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A30" s="55" t="s">
         <v>61</v>
       </c>
       <c r="B30" s="55"/>
       <c r="C30" s="55"/>
-      <c r="D30" s="27">
-        <f>SUM(E30:L30)</f>
+      <c r="D30" s="26">
+        <f t="shared" ref="D30:L30" si="3">D18+D28+D29</f>
         <v>0</v>
       </c>
       <c r="E30" s="26">
-        <f>SUM(E20:E29)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F30" s="26">
-        <f>SUM(F20:F29)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G30" s="26">
-        <f>SUM(G20:G29)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H30" s="26">
-        <f>SUM(H20:H29)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I30" s="26">
-        <f>SUM(I20:I29)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J30" s="26">
-        <f>SUM(J20:J29)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K30" s="26">
-        <f>SUM(K20:K29)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L30" s="26">
-        <f>SUM(L20:L29)</f>
-        <v>0</v>
-      </c>
-      <c r="M30" s="16"/>
-      <c r="N30" s="20"/>
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="M30" s="16">
+        <f>SUM(M18,M28,M29)</f>
+        <v>0</v>
+      </c>
+      <c r="N30" s="21"/>
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
       <c r="Q30" s="3"/>
@@ -2492,42 +2489,23 @@
       <c r="U30" s="3"/>
       <c r="V30" s="3"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A31" s="59" t="s">
+    <row r="31" spans="1:22" ht="15" x14ac:dyDescent="0.25">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="B31" s="59"/>
-      <c r="C31" s="59"/>
-      <c r="D31" s="27">
-        <f>SUM(E31:L31)</f>
-        <v>0</v>
-      </c>
-      <c r="E31" s="25">
-        <v>0</v>
-      </c>
-      <c r="F31" s="25">
-        <v>0</v>
-      </c>
-      <c r="G31" s="25">
-        <v>0</v>
-      </c>
-      <c r="H31" s="25">
-        <v>0</v>
-      </c>
-      <c r="I31" s="25">
-        <v>0</v>
-      </c>
-      <c r="J31" s="25">
-        <v>0</v>
-      </c>
-      <c r="K31" s="25">
-        <v>0</v>
-      </c>
-      <c r="L31" s="25">
-        <v>0</v>
-      </c>
-      <c r="M31" s="14"/>
-      <c r="N31" s="24"/>
+      <c r="K31" s="56"/>
+      <c r="L31" s="56"/>
+      <c r="M31" s="56"/>
+      <c r="N31" s="56"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
       <c r="Q31" s="3"/>
@@ -2537,50 +2515,25 @@
       <c r="U31" s="3"/>
       <c r="V31" s="3"/>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A32" s="56" t="s">
+    <row r="32" spans="1:22" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A32" s="3"/>
+      <c r="B32" s="57" t="s">
         <v>63</v>
       </c>
-      <c r="B32" s="56"/>
-      <c r="C32" s="56"/>
-      <c r="D32" s="26">
-        <f>D18+D30+D31</f>
-        <v>0</v>
-      </c>
-      <c r="E32" s="26">
-        <f>E18+E30+E31</f>
-        <v>0</v>
-      </c>
-      <c r="F32" s="26">
-        <f>F18+F30+F31</f>
-        <v>0</v>
-      </c>
-      <c r="G32" s="26">
-        <f>G18+G30+G31</f>
-        <v>0</v>
-      </c>
-      <c r="H32" s="26">
-        <f>H18+H30+H31</f>
-        <v>0</v>
-      </c>
-      <c r="I32" s="26">
-        <f>I18+I30+I31</f>
-        <v>0</v>
-      </c>
-      <c r="J32" s="26">
-        <f>J18+J30+J31</f>
-        <v>0</v>
-      </c>
-      <c r="K32" s="26">
-        <f>K18+K30+K31</f>
-        <v>0</v>
-      </c>
-      <c r="L32" s="26">
-        <f>L18+L30+L31</f>
-        <v>0</v>
-      </c>
-      <c r="M32" s="16"/>
-      <c r="N32" s="21"/>
+      <c r="C32" s="57"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="57" t="s">
+        <v>64</v>
+      </c>
+      <c r="K32" s="57"/>
+      <c r="L32" s="57"/>
+      <c r="M32" s="57"/>
+      <c r="N32" s="57"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
@@ -2590,23 +2543,25 @@
       <c r="U32" s="3"/>
       <c r="V32" s="3"/>
     </row>
-    <row r="33" spans="1:22" ht="15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
+      <c r="B33" s="52" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="52"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="57" t="s">
-        <v>64</v>
-      </c>
-      <c r="K33" s="57"/>
-      <c r="L33" s="57"/>
-      <c r="M33" s="57"/>
-      <c r="N33" s="57"/>
+      <c r="J33" s="52" t="s">
+        <v>66</v>
+      </c>
+      <c r="K33" s="52"/>
+      <c r="L33" s="52"/>
+      <c r="M33" s="52"/>
+      <c r="N33" s="52"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
@@ -2616,78 +2571,20 @@
       <c r="U33" s="3"/>
       <c r="V33" s="3"/>
     </row>
-    <row r="34" spans="1:22" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A34" s="3"/>
-      <c r="B34" s="58" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" s="58"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="58" t="s">
-        <v>66</v>
-      </c>
-      <c r="K34" s="58"/>
-      <c r="L34" s="58"/>
-      <c r="M34" s="58"/>
-      <c r="N34" s="58"/>
-      <c r="O34" s="3"/>
-      <c r="P34" s="3"/>
-      <c r="Q34" s="3"/>
-      <c r="R34" s="3"/>
-      <c r="S34" s="3"/>
-      <c r="T34" s="3"/>
-      <c r="U34" s="3"/>
-      <c r="V34" s="3"/>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A35" s="3"/>
-      <c r="B35" s="52" t="s">
-        <v>67</v>
-      </c>
-      <c r="C35" s="52"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
-      <c r="J35" s="52" t="s">
-        <v>68</v>
-      </c>
-      <c r="K35" s="52"/>
-      <c r="L35" s="52"/>
-      <c r="M35" s="52"/>
-      <c r="N35" s="52"/>
-      <c r="O35" s="3"/>
-      <c r="P35" s="3"/>
-      <c r="Q35" s="3"/>
-      <c r="R35" s="3"/>
-      <c r="S35" s="3"/>
-      <c r="T35" s="3"/>
-      <c r="U35" s="3"/>
-      <c r="V35" s="3"/>
-    </row>
   </sheetData>
-  <mergeCells count="48">
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="J35:N35"/>
+  <mergeCells count="46">
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="J33:N33"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="J33:N33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="J34:N34"/>
-    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="J31:N31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="J32:N32"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="A12:N12"/>
     <mergeCell ref="B13:C13"/>

</xml_diff>

<commit_message>
Updated vietnamese text in m4b1 report that should be in english
</commit_message>
<xml_diff>
--- a/api/templates/xpert_m4b1_patients/en.xlsx
+++ b/api/templates/xpert_m4b1_patients/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\xpert_m4b1_patients\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB16FAB-483A-46D1-B0FA-6A4E320430C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC8EAD26-9772-45B7-876B-66F435DC7D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B124328-57BC-4FCF-919D-A7394F83025A}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0B124328-57BC-4FCF-919D-A7394F83025A}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -79,9 +79,6 @@
     <t>Total number of test people</t>
   </si>
   <si>
-    <t>Phân loại kết quả</t>
-  </si>
-  <si>
     <t>Active screening/other</t>
   </si>
   <si>
@@ -264,6 +261,9 @@
   </si>
   <si>
     <t>Trace</t>
+  </si>
+  <si>
+    <t>Results Categories</t>
   </si>
 </sst>
 </file>
@@ -599,6 +599,109 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -613,109 +716,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1259,12 +1259,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="A1" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -1287,12 +1287,12 @@
       <c r="V1" s="3"/>
     </row>
     <row r="2" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -1313,22 +1313,22 @@
       <c r="V2" s="3"/>
     </row>
     <row r="3" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
-      <c r="K3" s="31"/>
-      <c r="L3" s="31"/>
-      <c r="M3" s="31"/>
-      <c r="N3" s="31"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="57"/>
+      <c r="N3" s="57"/>
       <c r="O3" s="4"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
@@ -1339,22 +1339,22 @@
       <c r="V3" s="3"/>
     </row>
     <row r="4" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="32"/>
-      <c r="M4" s="32"/>
-      <c r="N4" s="32"/>
+      <c r="A4" s="58" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="58"/>
       <c r="O4" s="5"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
@@ -1365,28 +1365,28 @@
       <c r="V4" s="3"/>
     </row>
     <row r="5" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
       <c r="F5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="34" t="s">
-        <v>70</v>
-      </c>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="34"/>
-      <c r="N5" s="34"/>
+      <c r="G5" s="53" t="s">
+        <v>69</v>
+      </c>
+      <c r="H5" s="53"/>
+      <c r="I5" s="53"/>
+      <c r="J5" s="53"/>
+      <c r="K5" s="53"/>
+      <c r="L5" s="53"/>
+      <c r="M5" s="53"/>
+      <c r="N5" s="53"/>
       <c r="O5" s="3"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
@@ -1401,28 +1401,28 @@
         <v>6</v>
       </c>
       <c r="B6" s="28"/>
-      <c r="C6" s="33" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
+      <c r="C6" s="52" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
       <c r="F6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="34" t="s">
-        <v>71</v>
-      </c>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
+      <c r="G6" s="53" t="s">
+        <v>70</v>
+      </c>
+      <c r="H6" s="53"/>
+      <c r="I6" s="53"/>
       <c r="J6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="K6" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34"/>
-      <c r="N6" s="34"/>
+      <c r="K6" s="53" t="s">
+        <v>71</v>
+      </c>
+      <c r="L6" s="53"/>
+      <c r="M6" s="53"/>
+      <c r="N6" s="53"/>
       <c r="O6" s="3"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="3"/>
@@ -1433,21 +1433,21 @@
       <c r="V6" s="3"/>
     </row>
     <row r="7" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33"/>
+      <c r="B7" s="52"/>
+      <c r="C7" s="52"/>
       <c r="D7" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="35" t="s">
+      <c r="G7" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
+      <c r="H7" s="54"/>
+      <c r="I7" s="54"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
@@ -1463,29 +1463,29 @@
       <c r="V7" s="3"/>
     </row>
     <row r="8" spans="1:24" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="37" t="s">
+      <c r="B8" s="43"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="40" t="s">
+      <c r="E8" s="47" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="47"/>
+      <c r="G8" s="47"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="47"/>
+      <c r="J8" s="47"/>
+      <c r="K8" s="47"/>
+      <c r="L8" s="47"/>
+      <c r="M8" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="40"/>
-      <c r="K8" s="40"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="42" t="s">
+      <c r="N8" s="47" t="s">
         <v>15</v>
-      </c>
-      <c r="N8" s="40" t="s">
-        <v>16</v>
       </c>
       <c r="O8" s="8"/>
       <c r="P8" s="3"/>
@@ -1497,30 +1497,30 @@
       <c r="V8" s="3"/>
     </row>
     <row r="9" spans="1:24" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="41" t="s">
+      <c r="A9" s="43"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="48" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="41" t="s">
+      <c r="G9" s="48"/>
+      <c r="H9" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="41"/>
-      <c r="H9" s="41" t="s">
+      <c r="I9" s="48"/>
+      <c r="J9" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="41"/>
-      <c r="J9" s="41" t="s">
-        <v>20</v>
-      </c>
-      <c r="K9" s="41"/>
-      <c r="L9" s="41" t="s">
-        <v>73</v>
-      </c>
-      <c r="M9" s="43"/>
-      <c r="N9" s="40"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="48" t="s">
+        <v>72</v>
+      </c>
+      <c r="M9" s="50"/>
+      <c r="N9" s="47"/>
       <c r="O9" s="8"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
@@ -1531,32 +1531,32 @@
       <c r="V9" s="3"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A10" s="36"/>
-      <c r="B10" s="36"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="41"/>
+      <c r="A10" s="43"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="48"/>
       <c r="F10" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="9" t="s">
-        <v>22</v>
-      </c>
       <c r="H10" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="I10" s="9" t="s">
-        <v>22</v>
-      </c>
       <c r="J10" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="L10" s="41"/>
-      <c r="M10" s="44"/>
-      <c r="N10" s="40"/>
+        <v>39</v>
+      </c>
+      <c r="L10" s="48"/>
+      <c r="M10" s="51"/>
+      <c r="N10" s="47"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
@@ -1567,41 +1567,41 @@
       <c r="V10" s="3"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A11" s="36"/>
-      <c r="B11" s="36"/>
-      <c r="C11" s="36"/>
+      <c r="A11" s="43"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
       <c r="D11" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="F11" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="G11" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="H11" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="I11" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="J11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="J11" s="13" t="s">
+      <c r="K11" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="L11" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="L11" s="13" t="s">
+      <c r="M11" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="M11" s="13" t="s">
+      <c r="N11" s="13" t="s">
         <v>32</v>
-      </c>
-      <c r="N11" s="13" t="s">
-        <v>33</v>
       </c>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1613,22 +1613,22 @@
       <c r="V11" s="3"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A12" s="46" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="46"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="46"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="46"/>
-      <c r="I12" s="46"/>
-      <c r="J12" s="46"/>
-      <c r="K12" s="46"/>
-      <c r="L12" s="46"/>
-      <c r="M12" s="46"/>
-      <c r="N12" s="46"/>
+      <c r="A12" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="37"/>
+      <c r="L12" s="37"/>
+      <c r="M12" s="37"/>
+      <c r="N12" s="37"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
@@ -1643,10 +1643,10 @@
       <c r="A13" s="24">
         <v>1</v>
       </c>
-      <c r="B13" s="47" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="47"/>
+      <c r="B13" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="38"/>
       <c r="D13" s="27">
         <f>SUM(E13:L13)</f>
         <v>0</v>
@@ -1690,10 +1690,10 @@
       <c r="A14" s="24">
         <v>2</v>
       </c>
-      <c r="B14" s="47" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="47"/>
+      <c r="B14" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="38"/>
       <c r="D14" s="27">
         <f>SUM(E14:L14)</f>
         <v>0</v>
@@ -1737,10 +1737,10 @@
       <c r="A15" s="24">
         <v>3</v>
       </c>
-      <c r="B15" s="47" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="47"/>
+      <c r="B15" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="38"/>
       <c r="D15" s="27">
         <f>SUM(E15:L15)</f>
         <v>0</v>
@@ -1781,14 +1781,14 @@
       <c r="V15" s="3"/>
     </row>
     <row r="16" spans="1:24" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="48">
+      <c r="A16" s="39">
         <v>4</v>
       </c>
-      <c r="B16" s="49" t="s">
+      <c r="B16" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="23" t="s">
         <v>38</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>39</v>
       </c>
       <c r="D16" s="27">
         <f>SUM(E16:L16)</f>
@@ -1830,10 +1830,10 @@
       <c r="V16" s="3"/>
     </row>
     <row r="17" spans="1:22" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="48"/>
-      <c r="B17" s="49"/>
+      <c r="A17" s="39"/>
+      <c r="B17" s="40"/>
       <c r="C17" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D17" s="27">
         <f>SUM(E17:L17)</f>
@@ -1875,11 +1875,11 @@
       <c r="V17" s="3"/>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A18" s="50" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="50"/>
-      <c r="C18" s="50"/>
+      <c r="A18" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="41"/>
+      <c r="C18" s="41"/>
       <c r="D18" s="26">
         <f>SUM(D13:D17)</f>
         <v>0</v>
@@ -1931,22 +1931,22 @@
       <c r="V18" s="3"/>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A19" s="51" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="51"/>
-      <c r="C19" s="51"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="51"/>
-      <c r="F19" s="51"/>
-      <c r="G19" s="51"/>
-      <c r="H19" s="51"/>
-      <c r="I19" s="51"/>
-      <c r="J19" s="51"/>
-      <c r="K19" s="51"/>
-      <c r="L19" s="51"/>
-      <c r="M19" s="51"/>
-      <c r="N19" s="51"/>
+      <c r="A19" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="42"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="42"/>
+      <c r="J19" s="42"/>
+      <c r="K19" s="42"/>
+      <c r="L19" s="42"/>
+      <c r="M19" s="42"/>
+      <c r="N19" s="42"/>
       <c r="O19" s="3"/>
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
@@ -1958,12 +1958,12 @@
     </row>
     <row r="20" spans="1:22" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="B20" s="45" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="45"/>
+      <c r="C20" s="30"/>
       <c r="D20" s="27">
         <f t="shared" ref="D20:D27" si="1">SUM(E20:L20)</f>
         <v>0</v>
@@ -2005,12 +2005,12 @@
     </row>
     <row r="21" spans="1:22" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="45" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="45"/>
+      <c r="C21" s="30"/>
       <c r="D21" s="27">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2052,12 +2052,12 @@
     </row>
     <row r="22" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="45" t="s">
-        <v>48</v>
-      </c>
-      <c r="C22" s="45"/>
+      <c r="C22" s="30"/>
       <c r="D22" s="27">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2099,12 +2099,12 @@
     </row>
     <row r="23" spans="1:22" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="B23" s="45" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" s="45"/>
+      <c r="C23" s="30"/>
       <c r="D23" s="27">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2146,12 +2146,12 @@
     </row>
     <row r="24" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="B24" s="45" t="s">
-        <v>52</v>
-      </c>
-      <c r="C24" s="45"/>
+      <c r="C24" s="30"/>
       <c r="D24" s="27">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2193,12 +2193,12 @@
     </row>
     <row r="25" spans="1:22" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="45" t="s">
-        <v>54</v>
-      </c>
-      <c r="C25" s="45"/>
+      <c r="C25" s="30"/>
       <c r="D25" s="27">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2240,12 +2240,12 @@
     </row>
     <row r="26" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="45" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26" s="45"/>
+      <c r="C26" s="30"/>
       <c r="D26" s="27">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2287,12 +2287,12 @@
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A27" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B27" s="53" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" s="45"/>
+      <c r="C27" s="30"/>
       <c r="D27" s="27">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2333,11 +2333,11 @@
       <c r="V27" s="3"/>
     </row>
     <row r="28" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="54" t="s">
-        <v>59</v>
-      </c>
-      <c r="B28" s="54"/>
-      <c r="C28" s="54"/>
+      <c r="A28" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
       <c r="D28" s="27">
         <f>SUM(E28:L28)</f>
         <v>0</v>
@@ -2389,11 +2389,11 @@
       <c r="V28" s="3"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A29" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="B29" s="58"/>
-      <c r="C29" s="58"/>
+      <c r="A29" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="36"/>
+      <c r="C29" s="36"/>
       <c r="D29" s="27">
         <f>SUM(E29:L29)</f>
         <v>0</v>
@@ -2434,11 +2434,11 @@
       <c r="V29" s="3"/>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A30" s="55" t="s">
-        <v>61</v>
-      </c>
-      <c r="B30" s="55"/>
-      <c r="C30" s="55"/>
+      <c r="A30" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="B30" s="33"/>
+      <c r="C30" s="33"/>
       <c r="D30" s="26">
         <f t="shared" ref="D30:L30" si="3">D18+D28+D29</f>
         <v>0</v>
@@ -2499,13 +2499,13 @@
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="56" t="s">
-        <v>62</v>
-      </c>
-      <c r="K31" s="56"/>
-      <c r="L31" s="56"/>
-      <c r="M31" s="56"/>
-      <c r="N31" s="56"/>
+      <c r="J31" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
+      <c r="M31" s="34"/>
+      <c r="N31" s="34"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
       <c r="Q31" s="3"/>
@@ -2517,23 +2517,23 @@
     </row>
     <row r="32" spans="1:22" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A32" s="3"/>
-      <c r="B32" s="57" t="s">
-        <v>63</v>
-      </c>
-      <c r="C32" s="57"/>
+      <c r="B32" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="35"/>
       <c r="D32" s="22"/>
       <c r="E32" s="22"/>
       <c r="F32" s="22"/>
       <c r="G32" s="22"/>
       <c r="H32" s="22"/>
       <c r="I32" s="22"/>
-      <c r="J32" s="57" t="s">
-        <v>64</v>
-      </c>
-      <c r="K32" s="57"/>
-      <c r="L32" s="57"/>
-      <c r="M32" s="57"/>
-      <c r="N32" s="57"/>
+      <c r="J32" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="K32" s="35"/>
+      <c r="L32" s="35"/>
+      <c r="M32" s="35"/>
+      <c r="N32" s="35"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
@@ -2545,23 +2545,23 @@
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A33" s="3"/>
-      <c r="B33" s="52" t="s">
-        <v>65</v>
-      </c>
-      <c r="C33" s="52"/>
+      <c r="B33" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="C33" s="29"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="52" t="s">
-        <v>66</v>
-      </c>
-      <c r="K33" s="52"/>
-      <c r="L33" s="52"/>
-      <c r="M33" s="52"/>
-      <c r="N33" s="52"/>
+      <c r="J33" s="29" t="s">
+        <v>65</v>
+      </c>
+      <c r="K33" s="29"/>
+      <c r="L33" s="29"/>
+      <c r="M33" s="29"/>
+      <c r="N33" s="29"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
@@ -2573,6 +2573,40 @@
     </row>
   </sheetData>
   <mergeCells count="46">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="G5:N5"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="A8:C11"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:L8"/>
+    <mergeCell ref="N8:N10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:N19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="J33:N33"/>
     <mergeCell ref="B24:C24"/>
@@ -2585,40 +2619,6 @@
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="J32:N32"/>
     <mergeCell ref="A29:C29"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A19:N19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="A8:C11"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:L8"/>
-    <mergeCell ref="N8:N10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="G5:N5"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>